<commit_message>
week 16 demo/exercise added
</commit_message>
<xml_diff>
--- a/Exercises/Presentations Assignment.xlsx
+++ b/Exercises/Presentations Assignment.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Trainings\2025-Freelance\2026 01 DotNet CHD Capgemini\CU-DotNet-Jan26-B4\Exercises\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Trainings\2025-Freelance\2026 01 DotNet CHD Capgemini\CU-DotNet-Jan26-B4 OLD\Exercises\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{567C040A-6E8F-401A-9D3B-4A72DA38ACBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BD48717-6135-415C-88F3-15DFCC0C6F34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{E9AF70C7-C994-4C29-A864-938A656EF003}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{E9AF70C7-C994-4C29-A864-938A656EF003}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="22 Apr" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="86">
   <si>
     <t>S.No</t>
   </si>
@@ -226,6 +227,72 @@
   </si>
   <si>
     <t>Indirect Recursion</t>
+  </si>
+  <si>
+    <t>Type Inference &amp; Dynamic Behavior</t>
+  </si>
+  <si>
+    <t>Core Object Model &amp; String Handling</t>
+  </si>
+  <si>
+    <t>Methods &amp; Parameterization</t>
+  </si>
+  <si>
+    <t>Debugging Fundamentals</t>
+  </si>
+  <si>
+    <t>Inheritance &amp; Polymorphism</t>
+  </si>
+  <si>
+    <t>Interfaces &amp; Generics</t>
+  </si>
+  <si>
+    <t>Exception Handling &amp; Resource Management</t>
+  </si>
+  <si>
+    <t>Collections, Delegates &amp; Concurrency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No pre written code </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Expecting pure coding based presentation </t>
+  </si>
+  <si>
+    <t>to explain the core concepts of the topic</t>
+  </si>
+  <si>
+    <t>Duration - At least 10 minutes</t>
+  </si>
+  <si>
+    <t>SNO</t>
+  </si>
+  <si>
+    <t>Topic</t>
+  </si>
+  <si>
+    <t>Arrays &amp; Lists</t>
+  </si>
+  <si>
+    <t>Unit Testing using Xunit</t>
+  </si>
+  <si>
+    <t>Dictionary and LINQ</t>
+  </si>
+  <si>
+    <t>LINQ operations and deferred execution</t>
+  </si>
+  <si>
+    <t>Abstract vs virtual / Overriding</t>
+  </si>
+  <si>
+    <t>Advanced C# 10 Language Features</t>
+  </si>
+  <si>
+    <t>C# Type System &amp; Coding Practices</t>
+  </si>
+  <si>
+    <t>Parsing, Conversion &amp; Project Referencing</t>
   </si>
 </sst>
 </file>
@@ -241,7 +308,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -251,6 +318,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -267,9 +340,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -590,7 +664,8 @@
     <col min="1" max="1" width="10.26953125" customWidth="1"/>
     <col min="2" max="2" width="31.90625" customWidth="1"/>
     <col min="3" max="3" width="23.26953125" customWidth="1"/>
-    <col min="6" max="6" width="15.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="0" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="15.90625" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
@@ -605,7 +680,7 @@
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
       <c r="D2" s="1" t="s">
@@ -619,7 +694,7 @@
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="2" t="s">
         <v>3</v>
       </c>
       <c r="D3" s="1" t="s">
@@ -633,7 +708,7 @@
       <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="2" t="s">
         <v>4</v>
       </c>
       <c r="D4" t="s">
@@ -643,11 +718,11 @@
         <v>52</v>
       </c>
     </row>
-    <row r="5" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="2" t="s">
         <v>5</v>
       </c>
       <c r="D5" t="s">
@@ -661,7 +736,7 @@
       <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D6" s="1" t="s">
@@ -675,7 +750,7 @@
       <c r="A7">
         <v>6</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D7" t="s">
@@ -689,7 +764,7 @@
       <c r="A8">
         <v>7</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D8" t="s">
@@ -703,7 +778,7 @@
       <c r="A9">
         <v>8</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D9" t="s">
@@ -717,7 +792,7 @@
       <c r="A10">
         <v>9</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D10" t="s">
@@ -731,7 +806,7 @@
       <c r="A11">
         <v>10</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D11" t="s">
@@ -745,7 +820,7 @@
       <c r="A12">
         <v>11</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D12" t="s">
@@ -759,7 +834,7 @@
       <c r="A13">
         <v>12</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="2" t="s">
         <v>13</v>
       </c>
       <c r="D13" t="s">
@@ -773,7 +848,7 @@
       <c r="A14">
         <v>13</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D14" t="s">
@@ -787,7 +862,7 @@
       <c r="A15">
         <v>14</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="2" t="s">
         <v>15</v>
       </c>
       <c r="D15" t="s">
@@ -801,7 +876,7 @@
       <c r="A16">
         <v>15</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="2" t="s">
         <v>16</v>
       </c>
       <c r="D16" s="1" t="s">
@@ -811,11 +886,11 @@
         <v>50</v>
       </c>
     </row>
-    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>16</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D17" t="s">
@@ -829,7 +904,7 @@
       <c r="A18">
         <v>17</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D18" t="s">
@@ -839,11 +914,11 @@
         <v>52</v>
       </c>
     </row>
-    <row r="19" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>18</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="2" t="s">
         <v>19</v>
       </c>
       <c r="D19" t="s">
@@ -857,7 +932,7 @@
       <c r="A20">
         <v>19</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="2" t="s">
         <v>20</v>
       </c>
       <c r="D20" t="s">
@@ -871,7 +946,7 @@
       <c r="A21">
         <v>20</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="2" t="s">
         <v>21</v>
       </c>
       <c r="D21" t="s">
@@ -885,7 +960,7 @@
       <c r="A22">
         <v>21</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="2" t="s">
         <v>22</v>
       </c>
       <c r="D22" t="s">
@@ -899,7 +974,7 @@
       <c r="A23">
         <v>22</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B23" s="2" t="s">
         <v>23</v>
       </c>
       <c r="D23" s="1" t="s">
@@ -913,7 +988,7 @@
       <c r="A24">
         <v>23</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="2" t="s">
         <v>24</v>
       </c>
       <c r="D24" t="s">
@@ -927,7 +1002,7 @@
       <c r="A25">
         <v>24</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="2" t="s">
         <v>25</v>
       </c>
       <c r="D25" t="s">
@@ -941,7 +1016,7 @@
       <c r="A26">
         <v>25</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="2" t="s">
         <v>26</v>
       </c>
       <c r="D26" t="s">
@@ -955,7 +1030,7 @@
       <c r="A27">
         <v>26</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B27" s="2" t="s">
         <v>27</v>
       </c>
       <c r="D27" t="s">
@@ -969,7 +1044,7 @@
       <c r="A28">
         <v>27</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B28" s="2" t="s">
         <v>28</v>
       </c>
       <c r="D28" s="1" t="s">
@@ -983,7 +1058,7 @@
       <c r="A29">
         <v>28</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B29" s="2" t="s">
         <v>29</v>
       </c>
       <c r="D29" t="s">
@@ -997,7 +1072,7 @@
       <c r="A30">
         <v>29</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B30" s="2" t="s">
         <v>30</v>
       </c>
       <c r="D30" t="s">
@@ -1011,7 +1086,7 @@
       <c r="A31">
         <v>30</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B31" s="2" t="s">
         <v>31</v>
       </c>
       <c r="D31" t="s">
@@ -1021,11 +1096,11 @@
         <v>51</v>
       </c>
     </row>
-    <row r="32" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>31</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B32" s="2" t="s">
         <v>32</v>
       </c>
       <c r="D32" t="s">
@@ -1039,7 +1114,7 @@
       <c r="A33">
         <v>32</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B33" s="2" t="s">
         <v>33</v>
       </c>
       <c r="D33" t="s">
@@ -1053,7 +1128,7 @@
       <c r="A34">
         <v>33</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B34" s="2" t="s">
         <v>34</v>
       </c>
       <c r="D34" t="s">
@@ -1067,7 +1142,7 @@
       <c r="A35">
         <v>34</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B35" s="2" t="s">
         <v>35</v>
       </c>
       <c r="D35" t="s">
@@ -1081,7 +1156,7 @@
       <c r="A36">
         <v>35</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B36" s="2" t="s">
         <v>36</v>
       </c>
       <c r="D36" t="s">
@@ -1091,11 +1166,11 @@
         <v>56</v>
       </c>
     </row>
-    <row r="37" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>36</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B37" s="2" t="s">
         <v>37</v>
       </c>
       <c r="D37" t="s">
@@ -1105,11 +1180,11 @@
         <v>57</v>
       </c>
     </row>
-    <row r="38" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>37</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B38" s="2" t="s">
         <v>38</v>
       </c>
       <c r="D38" t="s">
@@ -1119,11 +1194,11 @@
         <v>58</v>
       </c>
     </row>
-    <row r="39" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>38</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B39" s="2" t="s">
         <v>39</v>
       </c>
       <c r="D39" t="s">
@@ -1137,7 +1212,7 @@
       <c r="A40">
         <v>39</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B40" s="2" t="s">
         <v>40</v>
       </c>
       <c r="D40" t="s">
@@ -1151,7 +1226,7 @@
       <c r="A41">
         <v>40</v>
       </c>
-      <c r="B41" t="s">
+      <c r="B41" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D41" t="s">
@@ -1165,7 +1240,7 @@
       <c r="A42">
         <v>41</v>
       </c>
-      <c r="B42" t="s">
+      <c r="B42" s="2" t="s">
         <v>42</v>
       </c>
       <c r="D42" t="s">
@@ -1175,11 +1250,11 @@
         <v>62</v>
       </c>
     </row>
-    <row r="43" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>42</v>
       </c>
-      <c r="B43" t="s">
+      <c r="B43" s="2" t="s">
         <v>43</v>
       </c>
       <c r="D43" t="s">
@@ -1193,7 +1268,7 @@
       <c r="A44">
         <v>43</v>
       </c>
-      <c r="B44" t="s">
+      <c r="B44" s="2" t="s">
         <v>44</v>
       </c>
       <c r="D44" s="1" t="s">
@@ -1201,6 +1276,395 @@
       </c>
       <c r="F44" t="s">
         <v>52</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42A4E316-0BFA-4F6B-B046-6EF460F9BAD3}">
+  <dimension ref="A1:E33"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="27.36328125" customWidth="1"/>
+    <col min="3" max="3" width="38.54296875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E3" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" t="s">
+        <v>78</v>
+      </c>
+      <c r="E4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C6" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C14" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C15" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C17" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C18" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C19" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C20" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C21" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C22" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C23" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C24" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C25" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C26" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C27" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C28" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C29" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C30" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C31" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C33" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
week 16 demo added
</commit_message>
<xml_diff>
--- a/Exercises/Presentations Assignment.xlsx
+++ b/Exercises/Presentations Assignment.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Trainings\2025-Freelance\2026 01 DotNet CHD Capgemini\CU-DotNet-Jan26-B4 OLD\Exercises\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Trainings\2025-Freelance\2026 01 DotNet CHD Capgemini\CU-DotNet-Jan26-B4\Exercises\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BD48717-6135-415C-88F3-15DFCC0C6F34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83702A69-CA84-4C55-8695-5B419577C54C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{E9AF70C7-C994-4C29-A864-938A656EF003}"/>
   </bookViews>
@@ -286,13 +286,13 @@
     <t>Abstract vs virtual / Overriding</t>
   </si>
   <si>
-    <t>Advanced C# 10 Language Features</t>
-  </si>
-  <si>
     <t>C# Type System &amp; Coding Practices</t>
   </si>
   <si>
     <t>Parsing, Conversion &amp; Project Referencing</t>
+  </si>
+  <si>
+    <t>Advanced C# 12 Language Features</t>
   </si>
 </sst>
 </file>
@@ -328,7 +328,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -336,14 +336,32 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1289,17 +1307,17 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="27.36328125" customWidth="1"/>
-    <col min="3" max="3" width="38.54296875" customWidth="1"/>
+    <col min="3" max="3" width="43.1796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+      <c r="A1" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="3" t="s">
         <v>77</v>
       </c>
       <c r="E1" t="s">
@@ -1307,27 +1325,27 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2">
+      <c r="A2" s="3">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C2" t="s">
-        <v>84</v>
+      <c r="C2" s="3" t="s">
+        <v>83</v>
       </c>
       <c r="E2" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A3">
+      <c r="A3" s="3">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="3" t="s">
         <v>64</v>
       </c>
       <c r="E3" t="s">
@@ -1335,13 +1353,13 @@
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A4">
+      <c r="A4" s="3">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="3" t="s">
         <v>78</v>
       </c>
       <c r="E4" t="s">
@@ -1349,321 +1367,321 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A5">
+      <c r="A5" s="3">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="3" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A6">
+      <c r="A6" s="3">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="3" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A7">
+      <c r="A7" s="3">
         <v>6</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="3" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" s="3">
+        <v>7</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9" s="3">
+        <v>8</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10" s="3">
+        <v>9</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11" s="3">
+        <v>10</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A12" s="3">
+        <v>11</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A13" s="3">
+        <v>12</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A14" s="3">
+        <v>13</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A15" s="3">
+        <v>14</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C15" s="3" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" s="2" t="s">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A16" s="3">
+        <v>15</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" s="3">
         <v>16</v>
       </c>
-      <c r="C8" t="s">
+      <c r="B17" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A18" s="3">
+        <v>17</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A19" s="3">
+        <v>18</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A20" s="3">
+        <v>19</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A21" s="3">
+        <v>20</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A22" s="3">
+        <v>21</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A23" s="3">
+        <v>22</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A24" s="3">
+        <v>23</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C24" s="3" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C9" t="s">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A25" s="3">
+        <v>24</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C25" s="3" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" s="2" t="s">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A26" s="3">
+        <v>25</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A27" s="3">
+        <v>26</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A28" s="3">
+        <v>27</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A29" s="3">
+        <v>28</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A30" s="3">
+        <v>29</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A31" s="3">
+        <v>30</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A32" s="3">
         <v>31</v>
       </c>
-      <c r="C10" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C11" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C12" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C13" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C14" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A15">
-        <v>14</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C15" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A16">
+      <c r="B32" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A33" s="3">
+        <v>32</v>
+      </c>
+      <c r="B33" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C16" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A17">
-        <v>16</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C17" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A18">
-        <v>17</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C18" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A19">
-        <v>18</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C19" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A20">
-        <v>19</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C20" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A21">
-        <v>20</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C21" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A22">
-        <v>21</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C22" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A23">
-        <v>22</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C23" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A24">
-        <v>23</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C24" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A25">
-        <v>24</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C25" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A26">
-        <v>25</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C26" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A27">
-        <v>26</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C27" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A28">
-        <v>27</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C28" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A29">
-        <v>28</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C29" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A30">
-        <v>29</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C30" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A31">
-        <v>30</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C31" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A32">
-        <v>31</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C32" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A33">
-        <v>32</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C33" t="s">
+      <c r="C33" s="3" t="s">
         <v>71</v>
       </c>
     </row>

</xml_diff>